<commit_message>
sql qquery generator script changes
</commit_message>
<xml_diff>
--- a/Output.xlsx
+++ b/Output.xlsx
@@ -453,12 +453,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SELECT AVG(CASE WHEN age = 30 THEN salary END) as [Avg_Salary_Of_30],        AVG(CASE WHEN age = 35 THEN salary END) as [Avg_Salary_Of_35],        AVG(CASE WHEN age = 25 THEN salary END) as [Avg_Salary_Of_25] FROM Employee.dbo.Employee_Salary</t>
+          <t>SELECT AVG([30]) AS AvgSalary30, AVG([35]) AS AvgSalary35, AVG([25]) AS AvgSalary25 FROM  (SELECT age, salary  FROM Employee.dbo.Employee_Salary) AS SourceTable PIVOT (  AVG(salary)  FOR age IN ([30], [35], [25]) ) AS PivotTable;</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>content='A summary of different scenarios where data manipulation, analysis, and interpretation is needed through calculations, trends identification, pivot functions, data extraction and filtering based on age, salaries, and other variables.' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 38, 'prompt_tokens': 53, 'total_tokens': 91, 'completion_tokens_details': {'accepted_prediction_tokens': 0, 'audio_tokens': 0, 'reasoning_tokens': 0, 'rejected_prediction_tokens': 0}, 'prompt_tokens_details': {'audio_tokens': 0, 'cached_tokens': 0}}, 'model_name': 'gpt-4', 'system_fingerprint': None, 'id': 'chatcmpl-BXU40eTPul9B7vlS4brxdHPzExOxn', 'service_tier': None, 'finish_reason': 'stop', 'logprobs': None, 'content_filter_results': {}} id='run--f72239a5-1a1a-40fd-9c69-48bcbd2fda25-0' usage_metadata={'input_tokens': 53, 'output_tokens': 38, 'total_tokens': 91, 'input_token_details': {'audio': 0, 'cache_read': 0}, 'output_token_details': {'audio': 0, 'reasoning': 0}}</t>
+          <t>content='A summarized instruction to generate a pivot table report that shows the average incomes of people in the age groups of 25, 30, and 35.' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 31, 'prompt_tokens': 53, 'total_tokens': 84, 'completion_tokens_details': {'accepted_prediction_tokens': 0, 'audio_tokens': 0, 'reasoning_tokens': 0, 'rejected_prediction_tokens': 0}, 'prompt_tokens_details': {'audio_tokens': 0, 'cached_tokens': 0}}, 'model_name': 'gpt-4', 'system_fingerprint': None, 'id': 'chatcmpl-BXrNVMvisCxAFThnewBDQZHttJyVm', 'service_tier': None, 'finish_reason': 'stop', 'logprobs': None, 'content_filter_results': {}} id='run--0ba2cb03-775b-499e-819b-abfdc7061250-0' usage_metadata={'input_tokens': 53, 'output_tokens': 31, 'total_tokens': 84, 'input_token_details': {'audio': 0, 'cache_read': 0}, 'output_token_details': {'audio': 0, 'reasoning': 0}}</t>
         </is>
       </c>
     </row>
@@ -470,12 +470,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SELECT * FROM Employee.dbo.Employee_Salary</t>
+          <t>SELECT [id], [name], [age], [salary], [hire_date], [hire_timestamp] FROM [Employee.dbo.Employee_Salary]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>content="As an AI, I don't have access to any physical or digital sheet. Please provide the prompts you want me to explain." additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 26, 'prompt_tokens': 52, 'total_tokens': 78, 'completion_tokens_details': {'accepted_prediction_tokens': 0, 'audio_tokens': 0, 'reasoning_tokens': 0, 'rejected_prediction_tokens': 0}, 'prompt_tokens_details': {'audio_tokens': 0, 'cached_tokens': 0}}, 'model_name': 'gpt-4', 'system_fingerprint': None, 'id': 'chatcmpl-BXU4ApmbPn2nJgcJiQrothexst0Ot', 'service_tier': None, 'finish_reason': 'stop', 'logprobs': None, 'content_filter_results': {}} id='run--2c264659-d07d-472e-b5c7-3792bc00b710-0' usage_metadata={'input_tokens': 52, 'output_tokens': 26, 'total_tokens': 78, 'input_token_details': {'audio': 0, 'cache_read': 0}, 'output_token_details': {'audio': 0, 'reasoning': 0}}</t>
+          <t>content="As an AI, I don't have access to any physical or digital sheet. Please provide the prompts you want me to explain." additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 26, 'prompt_tokens': 52, 'total_tokens': 78, 'completion_tokens_details': {'accepted_prediction_tokens': 0, 'audio_tokens': 0, 'reasoning_tokens': 0, 'rejected_prediction_tokens': 0}, 'prompt_tokens_details': {'audio_tokens': 0, 'cached_tokens': 0}}, 'model_name': 'gpt-4', 'system_fingerprint': None, 'id': 'chatcmpl-BXrNbC1sycOMaN2IX29a41rpX7Zho', 'service_tier': None, 'finish_reason': 'stop', 'logprobs': None, 'content_filter_results': {}} id='run--1f6be7aa-1f51-4dcf-8fbc-d4e6eda5f7fd-0' usage_metadata={'input_tokens': 52, 'output_tokens': 26, 'total_tokens': 78, 'input_token_details': {'audio': 0, 'cache_read': 0}, 'output_token_details': {'audio': 0, 'reasoning': 0}}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
end to end automation develpoment solution by sath_action_new_xpath
</commit_message>
<xml_diff>
--- a/Output.xlsx
+++ b/Output.xlsx
@@ -453,12 +453,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SELECT AVG([30]) AS AvgSalary30, AVG([35]) AS AvgSalary35, AVG([25]) AS AvgSalary25 FROM  (SELECT age, salary  FROM Employee.dbo.Employee_Salary) AS SourceTable PIVOT (  AVG(salary)  FOR age IN ([30], [35], [25]) ) AS PivotTable;</t>
+          <t>SELECT AVG(CASE WHEN age = 30 THEN salary ELSE 0 END) AS 'Average_Salary_Age_30', AVG(CASE WHEN age = 35 THEN salary ELSE 0 END) AS 'Average_Salary_Age_35', AVG(CASE WHEN age = 25 THEN salary ELSE 0 END) AS 'Average_Salary_Age_25' FROM Employee.dbo.Employee_Salary;</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>content='A summarized instruction to generate a pivot table report that shows the average incomes of people in the age groups of 25, 30, and 35.' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 31, 'prompt_tokens': 53, 'total_tokens': 84, 'completion_tokens_details': {'accepted_prediction_tokens': 0, 'audio_tokens': 0, 'reasoning_tokens': 0, 'rejected_prediction_tokens': 0}, 'prompt_tokens_details': {'audio_tokens': 0, 'cached_tokens': 0}}, 'model_name': 'gpt-4', 'system_fingerprint': None, 'id': 'chatcmpl-BXrNVMvisCxAFThnewBDQZHttJyVm', 'service_tier': None, 'finish_reason': 'stop', 'logprobs': None, 'content_filter_results': {}} id='run--0ba2cb03-775b-499e-819b-abfdc7061250-0' usage_metadata={'input_tokens': 53, 'output_tokens': 31, 'total_tokens': 84, 'input_token_details': {'audio': 0, 'cache_read': 0}, 'output_token_details': {'audio': 0, 'reasoning': 0}}</t>
+          <t>content='The prompts in the sheet ask for refining and categorizing data, summarizing the information, comparing and analyzing different data values, and managing data using various Excel functions such as pivot, SUM, COUNT, VLOOKUP etc.' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 45, 'prompt_tokens': 53, 'total_tokens': 98, 'completion_tokens_details': {'accepted_prediction_tokens': 0, 'audio_tokens': 0, 'reasoning_tokens': 0, 'rejected_prediction_tokens': 0}, 'prompt_tokens_details': {'audio_tokens': 0, 'cached_tokens': 0}}, 'model_name': 'gpt-4', 'system_fingerprint': None, 'finish_reason': 'stop', 'logprobs': None, 'content_filter_results': {}} id='run-43ddac4a-2d18-4ae5-8638-5c933c56ff57-0' usage_metadata={'input_tokens': 53, 'output_tokens': 45, 'total_tokens': 98, 'input_token_details': {'audio': 0, 'cache_read': 0}, 'output_token_details': {'audio': 0, 'reasoning': 0}}</t>
         </is>
       </c>
     </row>
@@ -475,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>content="As an AI, I don't have access to any physical or digital sheet. Please provide the prompts you want me to explain." additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 26, 'prompt_tokens': 52, 'total_tokens': 78, 'completion_tokens_details': {'accepted_prediction_tokens': 0, 'audio_tokens': 0, 'reasoning_tokens': 0, 'rejected_prediction_tokens': 0}, 'prompt_tokens_details': {'audio_tokens': 0, 'cached_tokens': 0}}, 'model_name': 'gpt-4', 'system_fingerprint': None, 'id': 'chatcmpl-BXrNbC1sycOMaN2IX29a41rpX7Zho', 'service_tier': None, 'finish_reason': 'stop', 'logprobs': None, 'content_filter_results': {}} id='run--1f6be7aa-1f51-4dcf-8fbc-d4e6eda5f7fd-0' usage_metadata={'input_tokens': 52, 'output_tokens': 26, 'total_tokens': 78, 'input_token_details': {'audio': 0, 'cache_read': 0}, 'output_token_details': {'audio': 0, 'reasoning': 0}}</t>
+          <t>content="As an AI, I don't have access to any physical or digital sheet. Please provide the prompts you want me to explain." additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 26, 'prompt_tokens': 52, 'total_tokens': 78, 'completion_tokens_details': {'accepted_prediction_tokens': 0, 'audio_tokens': 0, 'reasoning_tokens': 0, 'rejected_prediction_tokens': 0}, 'prompt_tokens_details': {'audio_tokens': 0, 'cached_tokens': 0}}, 'model_name': 'gpt-4', 'system_fingerprint': None, 'finish_reason': 'stop', 'logprobs': None, 'content_filter_results': {}} id='run-dc807fd3-b861-4860-a1b5-9a1503ffcd1e-0' usage_metadata={'input_tokens': 52, 'output_tokens': 26, 'total_tokens': 78, 'input_token_details': {'audio': 0, 'cache_read': 0}, 'output_token_details': {'audio': 0, 'reasoning': 0}}</t>
         </is>
       </c>
     </row>

</xml_diff>